<commit_message>
[add] Dados de dezembro para as tabelas
</commit_message>
<xml_diff>
--- a/datasources/datasources_renavam.xlsx
+++ b/datasources/datasources_renavam.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/murilotuvani/projects/br-fleet-analysis/datasources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1E36545D-3852-544F-A179-76A997585FED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394F2727-D909-EE48-BD8C-D9F2C8B6E11E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38760" yWindow="600" windowWidth="36780" windowHeight="17240" xr2:uid="{C52316A4-E197-2849-83D2-DD851507E09C}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26420" xr2:uid="{C52316A4-E197-2849-83D2-DD851507E09C}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="143">
   <si>
     <t>https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/94f84f90-4a96-4c47-93c8-22239245f4a0/download/i_frota_por_uf_municipio_marca_e_modelo_ano_maio_2025.zip</t>
   </si>
@@ -414,6 +414,60 @@
   </si>
   <si>
     <t>datasource_url</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/5a8a7f18-1fca-4ec2-813b-220062e73c30/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2015.rar</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/registro-nacional-de-veiculos-automotores-renavam/resource/5a8a7f18-1fca-4ec2-813b-220062e73c30</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/668484cc-79aa-458b-b378-95dbfbfe4968/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2016.rar</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/registro-nacional-de-veiculos-automotores-renavam/resource/668484cc-79aa-458b-b378-95dbfbfe4968</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/647cf4dd-6180-4029-b08f-ec14c37d15c0/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2017.rar</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/registro-nacional-de-veiculos-automotores-renavam/resource/647cf4dd-6180-4029-b08f-ec14c37d15c0?inner_span=True</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/47030eca-c5a3-423e-a377-1bf8226ec5f1/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2018.zip</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/registro-nacional-de-veiculos-automotores-renavam/resource/47030eca-c5a3-423e-a377-1bf8226ec5f1?inner_span=True</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/37055ff5-4aa3-4b73-a7b3-e0e9d5955279/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2025.zip</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/registro-nacional-de-veiculos-automotores-renavam/resource/37055ff5-4aa3-4b73-a7b3-e0e9d5955279?inner_span=True</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/57d4644e-fe02-441b-93dd-71550e24df9b/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2022.zip</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/registro-nacional-de-veiculos-automotores-renavam/resource/57d4644e-fe02-441b-93dd-71550e24df9b?inner_span=True</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/4869946e-9df5-4ffb-a543-498dd3ede6bb/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2021.zip</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/registro-nacional-de-veiculos-automotores-renavam/resource/4869946e-9df5-4ffb-a543-498dd3ede6bb?inner_span=True</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/0064d20c-2047-479c-a8be-82796740b639/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2020.zip</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/registro-nacional-de-veiculos-automotores-renavam/resource/0064d20c-2047-479c-a8be-82796740b639?inner_span=True</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/f4030775-1eb1-43a5-ad82-e5024d23db85/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2019.zip</t>
+  </si>
+  <si>
+    <t>https://dados.transportes.gov.br/dataset/registro-nacional-de-veiculos-automotores-renavam/resource/f4030775-1eb1-43a5-ad82-e5024d23db85?inner_span=True</t>
   </si>
 </sst>
 </file>
@@ -797,7 +851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68480DDE-2190-FA41-842C-3B0DACC332E8}">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="138.5" bestFit="1" customWidth="1"/>
@@ -839,711 +893,812 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
-        <v>45870</v>
+        <v>45992</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>134</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>45839</v>
+        <v>45870</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>45778</v>
+        <v>45839</v>
       </c>
       <c r="B6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>0</v>
+        <v>56</v>
+      </c>
+      <c r="C6" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B7" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B13" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B16" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B17" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>45413</v>
+        <v>45444</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>45383</v>
+        <v>45413</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>45352</v>
+        <v>45383</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>45323</v>
+        <v>45352</v>
       </c>
       <c r="B21" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
-        <v>45292</v>
+        <v>45323</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
-        <v>45261</v>
+        <v>45292</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
-        <v>45231</v>
+        <v>45261</v>
       </c>
       <c r="B24" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
-        <v>45200</v>
+        <v>45231</v>
       </c>
       <c r="B25" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
-        <v>45170</v>
+        <v>45200</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
-        <v>45139</v>
+        <v>45170</v>
       </c>
       <c r="B27" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
-        <v>45108</v>
+        <v>45139</v>
       </c>
       <c r="B28" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>45078</v>
+        <v>45108</v>
       </c>
       <c r="B29" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
-        <v>44927</v>
+        <v>45078</v>
       </c>
       <c r="B30" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
-        <v>44743</v>
+        <v>44927</v>
       </c>
       <c r="B31" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
-        <v>44562</v>
+        <v>44896</v>
       </c>
       <c r="B32" t="s">
-        <v>52</v>
+        <v>136</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>53</v>
+        <v>135</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
-        <v>44378</v>
+        <v>44743</v>
       </c>
       <c r="B33" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
-        <v>44197</v>
+        <v>44562</v>
       </c>
       <c r="B34" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
-        <v>44013</v>
+        <v>44531</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>138</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>67</v>
+        <v>137</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
-        <v>43831</v>
+        <v>44378</v>
       </c>
       <c r="B36" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
-        <v>43647</v>
+        <v>44197</v>
       </c>
       <c r="B37" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
-        <v>43466</v>
+        <v>44166</v>
       </c>
       <c r="B38" t="s">
-        <v>72</v>
+        <v>140</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>73</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
-        <v>43282</v>
+        <v>44013</v>
       </c>
       <c r="B39" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
-        <v>43101</v>
+        <v>43831</v>
       </c>
       <c r="B40" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
-        <v>42917</v>
+        <v>43800</v>
       </c>
       <c r="B41" t="s">
-        <v>79</v>
+        <v>142</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>78</v>
+        <v>141</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
-        <v>42736</v>
+        <v>43647</v>
       </c>
       <c r="B42" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
-        <v>42552</v>
+        <v>43466</v>
       </c>
       <c r="B43" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
-        <v>42370</v>
+        <v>43435</v>
       </c>
       <c r="B44" t="s">
-        <v>84</v>
+        <v>132</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>85</v>
+        <v>131</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
-        <v>42248</v>
+        <v>43282</v>
       </c>
       <c r="B45" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
-        <v>42217</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>121</v>
+        <v>43101</v>
+      </c>
+      <c r="B46" t="s">
+        <v>77</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
-        <v>42125</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>89</v>
+        <v>43070</v>
+      </c>
+      <c r="B47" t="s">
+        <v>130</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>90</v>
+        <v>129</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
-        <v>42278</v>
+        <v>42917</v>
       </c>
       <c r="B48" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
-        <v>42095</v>
+        <v>42736</v>
       </c>
       <c r="B49" t="s">
-        <v>94</v>
-      </c>
-      <c r="C49" t="s">
-        <v>93</v>
+        <v>81</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
-        <v>42064</v>
-      </c>
-      <c r="B50" t="s">
-        <v>95</v>
+        <v>42705</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>128</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>96</v>
+        <v>127</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
-        <v>42005</v>
+        <v>42552</v>
       </c>
       <c r="B51" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
-        <v>41974</v>
+        <v>42370</v>
       </c>
       <c r="B52" t="s">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
-        <v>41944</v>
-      </c>
-      <c r="B53" t="s">
-        <v>101</v>
-      </c>
-      <c r="C53" t="s">
-        <v>102</v>
+        <v>42339</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="2">
-        <v>41821</v>
+        <v>42248</v>
       </c>
       <c r="B54" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="2">
-        <v>41791</v>
-      </c>
-      <c r="B55" t="s">
-        <v>106</v>
-      </c>
-      <c r="C55" t="s">
-        <v>105</v>
+        <v>42217</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="2">
-        <v>41760</v>
-      </c>
-      <c r="B56" t="s">
-        <v>108</v>
+        <v>42125</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
-        <v>41671</v>
+        <v>42278</v>
       </c>
       <c r="B57" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>110</v>
+        <v>91</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
-        <v>41640</v>
+        <v>42095</v>
       </c>
       <c r="B58" t="s">
-        <v>112</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>111</v>
+        <v>94</v>
+      </c>
+      <c r="C58" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
-        <v>41609</v>
+        <v>42064</v>
       </c>
       <c r="B59" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="2">
-        <v>41579</v>
+        <v>42005</v>
       </c>
       <c r="B60" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
-        <v>41456</v>
+        <v>41974</v>
       </c>
       <c r="B61" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" s="2">
+        <v>41944</v>
+      </c>
+      <c r="B62" t="s">
+        <v>101</v>
+      </c>
+      <c r="C62" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="2">
+        <v>41821</v>
+      </c>
+      <c r="B63" t="s">
+        <v>104</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="2">
+        <v>41791</v>
+      </c>
+      <c r="B64" t="s">
+        <v>106</v>
+      </c>
+      <c r="C64" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" s="2">
+        <v>41760</v>
+      </c>
+      <c r="B65" t="s">
+        <v>108</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66" s="2">
+        <v>41671</v>
+      </c>
+      <c r="B66" t="s">
+        <v>109</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="2">
+        <v>41640</v>
+      </c>
+      <c r="B67" t="s">
+        <v>112</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="2">
+        <v>41609</v>
+      </c>
+      <c r="B68" t="s">
+        <v>114</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="2">
+        <v>41579</v>
+      </c>
+      <c r="B69" t="s">
+        <v>116</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="2">
+        <v>41456</v>
+      </c>
+      <c r="B70" t="s">
+        <v>118</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="2">
         <v>41395</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B71" t="s">
         <v>120</v>
       </c>
-      <c r="C62" s="1" t="s">
+      <c r="C71" s="1" t="s">
         <v>119</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C6" r:id="rId1" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/94f84f90-4a96-4c47-93c8-22239245f4a0/download/i_frota_por_uf_municipio_marca_e_modelo_ano_maio_2025.zip" xr:uid="{5707FF45-B52F-7941-A100-6C5BA0760877}"/>
-    <hyperlink ref="C7" r:id="rId2" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/22164b81-af61-440b-b02f-dc6bb7452002/download/i_frota_por_uf_municipio_marca_e_modelo_ano_abril_2025.zip" xr:uid="{C91BE1F1-F87E-F947-AC8C-35AEB028E440}"/>
-    <hyperlink ref="C8" r:id="rId3" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/61b71526-aff6-4517-9b65-43e251832b34/download/i_frota_por_uf_municipio_marca_e_modelo_ano_marco_2025.zip" xr:uid="{8CF92F89-E603-4E40-8920-B888AB464509}"/>
-    <hyperlink ref="C9" r:id="rId4" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/c95e5965-3501-4712-8788-a96c768cf81f/download/i_frota_por_uf_municipio_marca_e_modelo_ano_fevereiro_2025.zip" xr:uid="{E7900AE7-D4F2-0C4A-958C-42FFEF883B8B}"/>
-    <hyperlink ref="C10" r:id="rId5" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/36c0562e-1fc1-49c9-9a8d-c805d29e87cd/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2025.zip" xr:uid="{11B272C2-A456-964A-9BB5-CC43DA7D988F}"/>
-    <hyperlink ref="C11" r:id="rId6" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/fac336c0-c30c-44b6-bd12-666eee01cce5/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2024.zip" xr:uid="{3B8931F9-1BF2-AA4B-ACD8-DA29E066F42E}"/>
-    <hyperlink ref="C12" r:id="rId7" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/276afdab-2f9e-47e4-8590-a12c81ce2fcd/download/i_frota_por_uf_municipio_marca_e_modelo_ano_novembro_2024.zip" xr:uid="{20A55D3F-C5AA-DD49-8AED-2C7328F54EC2}"/>
-    <hyperlink ref="C13" r:id="rId8" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/37094b43-2c8f-4fc7-91c6-3775115a0a1a/download/i_frota_por_uf_municipio_marca_e_modelo_ano_outubro_2024.zip" xr:uid="{8609CFE4-A98D-4D4C-902D-0761F4A89B53}"/>
-    <hyperlink ref="C14" r:id="rId9" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/40744050-dc2a-4165-bbfb-3e4f624f58c0/download/i_frota_por_uf_municipio_marca_e_modelo_ano_setembro_2024.zip" xr:uid="{CB2689CC-F159-C541-8D01-F63A104BF722}"/>
-    <hyperlink ref="C15" r:id="rId10" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/bddfba35-789f-4afa-8d5e-9707ebcef241/download/i_frota_por_uf_municipio_marca_e_modelo_ano_agosto_2024.zip" xr:uid="{958B3D16-54E9-E542-9397-D8D087EC0032}"/>
-    <hyperlink ref="C16" r:id="rId11" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/49963e10-546a-4d72-8269-1489f4e5f349/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2024.zip" xr:uid="{4B2AF3F0-4A61-5640-A666-9F424D33F130}"/>
-    <hyperlink ref="C17" r:id="rId12" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/29df629f-a955-4427-a819-097334df9c84/download/i_frota_por_uf_municipio_marca_e_modelo_ano_junho_2024.zip" xr:uid="{E3D6DF7F-0300-EB47-90F6-E1F60DD7E63A}"/>
-    <hyperlink ref="C18" r:id="rId13" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/cd5817d2-c8db-4c21-8282-1f31f944f34d/download/i_frota_por_uf_municipio_marca_e_modelo_ano_maio_2024.zip" xr:uid="{A530C541-8593-A340-9192-8859B23A9E71}"/>
-    <hyperlink ref="C19" r:id="rId14" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/37e79e91-6db2-47ce-8a7f-b1ab1a465add/download/i_frota_por_uf_municipio_marca_e_modelo_ano_abril_2024.zip" xr:uid="{477A169B-30AA-1E4E-AC7F-0904387C17A1}"/>
-    <hyperlink ref="C20" r:id="rId15" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/6dd78090-aab1-4005-9dcf-0e045beaf5dc/download/i_frota_por_uf_municipio_marca_e_modelo_ano_marco_2024.zip" xr:uid="{CC5DE5C9-3E54-C347-BF94-C442E18BACBC}"/>
-    <hyperlink ref="C21" r:id="rId16" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/d33173dd-48b1-42aa-b42b-be4ced118a8e/download/i_frota_por_uf_municipio_marca_e_modelo_ano_fevereiro_2024.zip" xr:uid="{7E256274-12AC-9A40-91ED-BCC6DDF8C390}"/>
-    <hyperlink ref="C22" r:id="rId17" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/2427ca95-ccb4-4711-be8f-369e8a4f3178/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2024.zip" xr:uid="{84338004-6D5E-014D-9CF0-BB0495328367}"/>
-    <hyperlink ref="C23" r:id="rId18" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/023bf4a1-89b9-4947-9b2b-864fc097338f/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2023.zip" xr:uid="{743C662F-8988-B24F-9F08-5B99FCF1D63F}"/>
-    <hyperlink ref="C24" r:id="rId19" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/c338b00f-98e2-4d12-8d4c-00c3bb9eab1a/download/i_frota_por_uf_municipio_marca_e_modelo_ano_novembro_2023.zip" xr:uid="{262D4D91-71EC-0844-8364-FFFBFC1A2F40}"/>
-    <hyperlink ref="C25" r:id="rId20" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/e5ca029e-ffb0-4f2f-8768-e360b5d16c89/download/i_frota_por_uf_municipio_marca_e_modelo_ano_outubro_2023.zip" xr:uid="{F92A40E6-78CD-574E-8F7F-DF862B89195D}"/>
-    <hyperlink ref="C26" r:id="rId21" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/0e630abc-1728-4b52-82fd-b576242bad75/download/i_frota_por_uf_municipio_marca_e_modelo_ano_setembro_2023.zip" xr:uid="{357B991D-D6FC-D64F-A60C-17730587E0CA}"/>
-    <hyperlink ref="C27" r:id="rId22" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/3c7f83ef-785b-4d4f-94f2-a33fd99ec24e/download/i_frota_por_uf_municipio_marca_e_modelo_ano_agosto_2023.zip" xr:uid="{0700CA72-0D57-6F4E-963F-F8241BACB463}"/>
-    <hyperlink ref="C28" r:id="rId23" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/ac39ebfb-9920-47b4-8a47-60a96b355b3f/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2023.zip" xr:uid="{F97895CF-90B5-E843-86E2-9F505695FAA4}"/>
-    <hyperlink ref="C29" r:id="rId24" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/a828304e-ade2-43bd-9841-d0a691f2dc34/download/i_frota_por_uf_municipio_marca_e_modelo_ano_junho_2023.zip" xr:uid="{999D3503-B0D5-B940-84BE-BB2613AE2A14}"/>
-    <hyperlink ref="C30" r:id="rId25" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/4f6b4c22-ba2d-4e06-8f40-387bf9391824/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2023.zip" xr:uid="{6E50D934-44C9-E741-B5F1-B3FB8C890EA6}"/>
-    <hyperlink ref="C31" r:id="rId26" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/a4e485a7-4c7e-4034-81ed-c08232185455/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2022.zip" xr:uid="{1B6E0C96-F506-EA4D-BDDA-3668981DB90C}"/>
-    <hyperlink ref="C32" r:id="rId27" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/5a8a6b0e-87bc-428b-a277-51bcfecab41e/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2022.zip" xr:uid="{ED36E3BC-2225-0241-8962-B939414D4DA5}"/>
-    <hyperlink ref="C33" r:id="rId28" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/7ab94c38-e682-4190-8108-79c9dc581769/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2021.zip" xr:uid="{9D8F22AD-07AE-8E4E-8E12-E93FB430C7F0}"/>
-    <hyperlink ref="C34" r:id="rId29" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/4f31e0f2-6f6e-4a88-bc0d-d6d00141224a/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2021.zip" xr:uid="{63BC83F5-6F25-1544-A244-ED309EC8DFEC}"/>
-    <hyperlink ref="C35" r:id="rId30" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/f685440e-0af9-4678-85ed-5f2c7d7d2b3f/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2020.zip" xr:uid="{7632F639-4275-E54C-86B6-F31760ED6486}"/>
-    <hyperlink ref="C36" r:id="rId31" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/9d5fe257-c63d-4ed7-aadf-6c99db6f7362/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2020.zip" xr:uid="{3946FC74-7C20-854F-BF99-769DE07B918F}"/>
-    <hyperlink ref="C37" r:id="rId32" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/13875e10-613d-4472-a818-f2de56da6d25/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2019.zip" xr:uid="{DC0EE5FD-8159-2948-BAE0-451A6AA28B0A}"/>
-    <hyperlink ref="C38" r:id="rId33" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/0c5c37de-cdd0-49d0-93c0-bd72f6c5ac8a/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2019.zip" xr:uid="{34CD241E-D23A-1440-8EA9-6BB0AD6A9040}"/>
-    <hyperlink ref="C39" r:id="rId34" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/d9fae7a7-ec08-4132-99d6-347d91573783/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2018.rar" xr:uid="{2BF5C3C0-59C1-B942-A1CF-FBCB127188D7}"/>
-    <hyperlink ref="C40" r:id="rId35" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/42eeb955-86bd-430f-a2d0-16b49bb1e0fa/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2018.rar" xr:uid="{459A7E06-E135-0D40-B39A-EA75EB67F41B}"/>
-    <hyperlink ref="C41" r:id="rId36" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/0e30e4f2-f8ca-4783-bd1d-a6952461bdc1/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2017.rar" xr:uid="{50AD2AA4-5B5E-5248-8C89-EC5D643EBE0D}"/>
-    <hyperlink ref="C42" r:id="rId37" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/81550327-2b16-4cf3-b8e0-d6000c6dbf42/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2017.rar" xr:uid="{314D69DA-0177-194F-ACF3-014B396F39F2}"/>
-    <hyperlink ref="C43" r:id="rId38" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/95f2a20b-c7cd-4146-9931-0460a87d2b7c/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2016.rar" xr:uid="{FEB8C29C-6FD4-334D-8F74-12D9414AEFAD}"/>
-    <hyperlink ref="C44" r:id="rId39" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/079e3a33-728f-468a-b435-5ea1be346e42/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2016.rar" xr:uid="{918F7FA8-4445-BA40-9491-2E6AC84544B7}"/>
-    <hyperlink ref="C45" r:id="rId40" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/58d1a29c-7c17-4ace-86e9-552f5e4f9644/download/i_frota_por_uf_municipio_marca_e_modelo_ano_setembro_2015.rar" xr:uid="{D9506705-92A1-FA48-987D-2D08081E85F2}"/>
-    <hyperlink ref="C46" r:id="rId41" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/d0db7133-2e02-45b1-ba9f-ec9375c7250d/download/i_frota_por_uf_municipio_marca_e_modelo_ano_agosto_2015.rar" xr:uid="{871DA683-A296-7B49-93AE-6FF668332080}"/>
-    <hyperlink ref="C47" r:id="rId42" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/124c530e-7212-4026-b874-e954ae32f08a/download/i_frota_por_uf_municipio_marca_e_modelo_ano_maio_2015.rar" xr:uid="{3BEA8807-31AB-B345-BF9B-6D455A8F9A8D}"/>
-    <hyperlink ref="C48" r:id="rId43" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/30293b59-f3ed-4b7e-beac-6255a98595ff/download/i_frota_por_uf_municipio_marca_e_modelo_ano_outubro_2015.rar" xr:uid="{D0E20417-0F4B-EF47-893D-62CA80C50D9E}"/>
-    <hyperlink ref="C50" r:id="rId44" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/1ced3149-49a1-4248-bcda-75d267e56059/download/i_frota_por_uf_municipio_marca_e_modelo_ano_marco_2015.rar" xr:uid="{D9248F29-E2EC-3442-928F-4D8ED7815325}"/>
-    <hyperlink ref="C51" r:id="rId45" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/93520344-d868-4e4f-afec-a295a5b09f52/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2015.rar" xr:uid="{67F18216-7680-AB49-B5FE-569D1FA8AD0D}"/>
-    <hyperlink ref="C52" r:id="rId46" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/f3b46afe-0ba1-452d-a04d-df23446161ca/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2014.zip" xr:uid="{07B73C55-8DA7-6F4D-9199-E73D20D4342B}"/>
-    <hyperlink ref="C54" r:id="rId47" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/73319382-e55d-422b-97fc-7127a37237a3/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2014.zip" xr:uid="{0E0D127C-3B25-284B-A195-BEC29EC9877C}"/>
-    <hyperlink ref="C56" r:id="rId48" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/5a4867ff-2453-4238-b440-885c835bc233/download/i_frota_por_uf_municipio_marca_e_modelo_ano_maio_2014.zip" xr:uid="{BC9A8E4E-AEBF-3D40-A856-36B368E6A0E7}"/>
-    <hyperlink ref="C57" r:id="rId49" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/1c199cdd-9581-4a07-a205-a7e378464717/download/i_frota_por_uf_municipio_marca_e_modelo_ano_fevereiro_2014.zip" xr:uid="{B4A42A7A-B149-4644-8E2D-77748F7BCFEB}"/>
-    <hyperlink ref="C58" r:id="rId50" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/cbcb4b9d-745d-42f7-89e4-b2eb6e55d320/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2014.zip" xr:uid="{543763BC-DAC0-6746-9C91-F2351B12BC27}"/>
-    <hyperlink ref="C59" r:id="rId51" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/086f527b-ba8c-40cf-bf37-d050978db888/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2013.zip" xr:uid="{7B49B406-BBF9-3449-B5D0-EA315FC8DEC2}"/>
-    <hyperlink ref="C60" r:id="rId52" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/1d89882c-da9e-4019-9711-c27919bb99d7/download/i_frota_por_uf_municipio_marca_e_modelo_ano_novembro_2013.zip" xr:uid="{36DF4B8B-2C67-E14E-BC44-91D8640C2BB1}"/>
-    <hyperlink ref="C61" r:id="rId53" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/60cd5ad4-d96b-46c8-9d81-30fc25cd163e/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2013.zip" xr:uid="{D202EEBF-FA2D-A948-8A27-AED2FEE897C0}"/>
-    <hyperlink ref="C62" r:id="rId54" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/e0d5ae22-bf42-447a-a788-2f6f1edf9705/download/i_frota_por_uf_municipio_marca_e_modelo_ano_maio_2013.zip" xr:uid="{D29B307C-D684-684D-B808-896574FA432D}"/>
-    <hyperlink ref="B46" r:id="rId55" xr:uid="{1A3D428E-E368-FB42-A8D4-DD387A74FB5C}"/>
-    <hyperlink ref="B47" r:id="rId56" xr:uid="{FF4AAA16-5B7E-4545-A83F-62ABEA4F564D}"/>
+    <hyperlink ref="C7" r:id="rId1" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/94f84f90-4a96-4c47-93c8-22239245f4a0/download/i_frota_por_uf_municipio_marca_e_modelo_ano_maio_2025.zip" xr:uid="{5707FF45-B52F-7941-A100-6C5BA0760877}"/>
+    <hyperlink ref="C8" r:id="rId2" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/22164b81-af61-440b-b02f-dc6bb7452002/download/i_frota_por_uf_municipio_marca_e_modelo_ano_abril_2025.zip" xr:uid="{C91BE1F1-F87E-F947-AC8C-35AEB028E440}"/>
+    <hyperlink ref="C9" r:id="rId3" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/61b71526-aff6-4517-9b65-43e251832b34/download/i_frota_por_uf_municipio_marca_e_modelo_ano_marco_2025.zip" xr:uid="{8CF92F89-E603-4E40-8920-B888AB464509}"/>
+    <hyperlink ref="C10" r:id="rId4" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/c95e5965-3501-4712-8788-a96c768cf81f/download/i_frota_por_uf_municipio_marca_e_modelo_ano_fevereiro_2025.zip" xr:uid="{E7900AE7-D4F2-0C4A-958C-42FFEF883B8B}"/>
+    <hyperlink ref="C11" r:id="rId5" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/36c0562e-1fc1-49c9-9a8d-c805d29e87cd/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2025.zip" xr:uid="{11B272C2-A456-964A-9BB5-CC43DA7D988F}"/>
+    <hyperlink ref="C12" r:id="rId6" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/fac336c0-c30c-44b6-bd12-666eee01cce5/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2024.zip" xr:uid="{3B8931F9-1BF2-AA4B-ACD8-DA29E066F42E}"/>
+    <hyperlink ref="C13" r:id="rId7" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/276afdab-2f9e-47e4-8590-a12c81ce2fcd/download/i_frota_por_uf_municipio_marca_e_modelo_ano_novembro_2024.zip" xr:uid="{20A55D3F-C5AA-DD49-8AED-2C7328F54EC2}"/>
+    <hyperlink ref="C14" r:id="rId8" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/37094b43-2c8f-4fc7-91c6-3775115a0a1a/download/i_frota_por_uf_municipio_marca_e_modelo_ano_outubro_2024.zip" xr:uid="{8609CFE4-A98D-4D4C-902D-0761F4A89B53}"/>
+    <hyperlink ref="C15" r:id="rId9" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/40744050-dc2a-4165-bbfb-3e4f624f58c0/download/i_frota_por_uf_municipio_marca_e_modelo_ano_setembro_2024.zip" xr:uid="{CB2689CC-F159-C541-8D01-F63A104BF722}"/>
+    <hyperlink ref="C16" r:id="rId10" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/bddfba35-789f-4afa-8d5e-9707ebcef241/download/i_frota_por_uf_municipio_marca_e_modelo_ano_agosto_2024.zip" xr:uid="{958B3D16-54E9-E542-9397-D8D087EC0032}"/>
+    <hyperlink ref="C17" r:id="rId11" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/49963e10-546a-4d72-8269-1489f4e5f349/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2024.zip" xr:uid="{4B2AF3F0-4A61-5640-A666-9F424D33F130}"/>
+    <hyperlink ref="C18" r:id="rId12" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/29df629f-a955-4427-a819-097334df9c84/download/i_frota_por_uf_municipio_marca_e_modelo_ano_junho_2024.zip" xr:uid="{E3D6DF7F-0300-EB47-90F6-E1F60DD7E63A}"/>
+    <hyperlink ref="C19" r:id="rId13" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/cd5817d2-c8db-4c21-8282-1f31f944f34d/download/i_frota_por_uf_municipio_marca_e_modelo_ano_maio_2024.zip" xr:uid="{A530C541-8593-A340-9192-8859B23A9E71}"/>
+    <hyperlink ref="C20" r:id="rId14" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/37e79e91-6db2-47ce-8a7f-b1ab1a465add/download/i_frota_por_uf_municipio_marca_e_modelo_ano_abril_2024.zip" xr:uid="{477A169B-30AA-1E4E-AC7F-0904387C17A1}"/>
+    <hyperlink ref="C21" r:id="rId15" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/6dd78090-aab1-4005-9dcf-0e045beaf5dc/download/i_frota_por_uf_municipio_marca_e_modelo_ano_marco_2024.zip" xr:uid="{CC5DE5C9-3E54-C347-BF94-C442E18BACBC}"/>
+    <hyperlink ref="C22" r:id="rId16" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/d33173dd-48b1-42aa-b42b-be4ced118a8e/download/i_frota_por_uf_municipio_marca_e_modelo_ano_fevereiro_2024.zip" xr:uid="{7E256274-12AC-9A40-91ED-BCC6DDF8C390}"/>
+    <hyperlink ref="C23" r:id="rId17" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/2427ca95-ccb4-4711-be8f-369e8a4f3178/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2024.zip" xr:uid="{84338004-6D5E-014D-9CF0-BB0495328367}"/>
+    <hyperlink ref="C24" r:id="rId18" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/023bf4a1-89b9-4947-9b2b-864fc097338f/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2023.zip" xr:uid="{743C662F-8988-B24F-9F08-5B99FCF1D63F}"/>
+    <hyperlink ref="C25" r:id="rId19" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/c338b00f-98e2-4d12-8d4c-00c3bb9eab1a/download/i_frota_por_uf_municipio_marca_e_modelo_ano_novembro_2023.zip" xr:uid="{262D4D91-71EC-0844-8364-FFFBFC1A2F40}"/>
+    <hyperlink ref="C26" r:id="rId20" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/e5ca029e-ffb0-4f2f-8768-e360b5d16c89/download/i_frota_por_uf_municipio_marca_e_modelo_ano_outubro_2023.zip" xr:uid="{F92A40E6-78CD-574E-8F7F-DF862B89195D}"/>
+    <hyperlink ref="C27" r:id="rId21" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/0e630abc-1728-4b52-82fd-b576242bad75/download/i_frota_por_uf_municipio_marca_e_modelo_ano_setembro_2023.zip" xr:uid="{357B991D-D6FC-D64F-A60C-17730587E0CA}"/>
+    <hyperlink ref="C28" r:id="rId22" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/3c7f83ef-785b-4d4f-94f2-a33fd99ec24e/download/i_frota_por_uf_municipio_marca_e_modelo_ano_agosto_2023.zip" xr:uid="{0700CA72-0D57-6F4E-963F-F8241BACB463}"/>
+    <hyperlink ref="C29" r:id="rId23" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/ac39ebfb-9920-47b4-8a47-60a96b355b3f/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2023.zip" xr:uid="{F97895CF-90B5-E843-86E2-9F505695FAA4}"/>
+    <hyperlink ref="C30" r:id="rId24" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/a828304e-ade2-43bd-9841-d0a691f2dc34/download/i_frota_por_uf_municipio_marca_e_modelo_ano_junho_2023.zip" xr:uid="{999D3503-B0D5-B940-84BE-BB2613AE2A14}"/>
+    <hyperlink ref="C31" r:id="rId25" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/4f6b4c22-ba2d-4e06-8f40-387bf9391824/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2023.zip" xr:uid="{6E50D934-44C9-E741-B5F1-B3FB8C890EA6}"/>
+    <hyperlink ref="C33" r:id="rId26" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/a4e485a7-4c7e-4034-81ed-c08232185455/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2022.zip" xr:uid="{1B6E0C96-F506-EA4D-BDDA-3668981DB90C}"/>
+    <hyperlink ref="C34" r:id="rId27" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/5a8a6b0e-87bc-428b-a277-51bcfecab41e/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2022.zip" xr:uid="{ED36E3BC-2225-0241-8962-B939414D4DA5}"/>
+    <hyperlink ref="C36" r:id="rId28" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/7ab94c38-e682-4190-8108-79c9dc581769/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2021.zip" xr:uid="{9D8F22AD-07AE-8E4E-8E12-E93FB430C7F0}"/>
+    <hyperlink ref="C37" r:id="rId29" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/4f31e0f2-6f6e-4a88-bc0d-d6d00141224a/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2021.zip" xr:uid="{63BC83F5-6F25-1544-A244-ED309EC8DFEC}"/>
+    <hyperlink ref="C39" r:id="rId30" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/f685440e-0af9-4678-85ed-5f2c7d7d2b3f/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2020.zip" xr:uid="{7632F639-4275-E54C-86B6-F31760ED6486}"/>
+    <hyperlink ref="C40" r:id="rId31" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/9d5fe257-c63d-4ed7-aadf-6c99db6f7362/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2020.zip" xr:uid="{3946FC74-7C20-854F-BF99-769DE07B918F}"/>
+    <hyperlink ref="C42" r:id="rId32" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/13875e10-613d-4472-a818-f2de56da6d25/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2019.zip" xr:uid="{DC0EE5FD-8159-2948-BAE0-451A6AA28B0A}"/>
+    <hyperlink ref="C43" r:id="rId33" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/0c5c37de-cdd0-49d0-93c0-bd72f6c5ac8a/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2019.zip" xr:uid="{34CD241E-D23A-1440-8EA9-6BB0AD6A9040}"/>
+    <hyperlink ref="C45" r:id="rId34" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/d9fae7a7-ec08-4132-99d6-347d91573783/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2018.rar" xr:uid="{2BF5C3C0-59C1-B942-A1CF-FBCB127188D7}"/>
+    <hyperlink ref="C46" r:id="rId35" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/42eeb955-86bd-430f-a2d0-16b49bb1e0fa/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2018.rar" xr:uid="{459A7E06-E135-0D40-B39A-EA75EB67F41B}"/>
+    <hyperlink ref="C48" r:id="rId36" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/0e30e4f2-f8ca-4783-bd1d-a6952461bdc1/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2017.rar" xr:uid="{50AD2AA4-5B5E-5248-8C89-EC5D643EBE0D}"/>
+    <hyperlink ref="C49" r:id="rId37" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/81550327-2b16-4cf3-b8e0-d6000c6dbf42/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2017.rar" xr:uid="{314D69DA-0177-194F-ACF3-014B396F39F2}"/>
+    <hyperlink ref="C51" r:id="rId38" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/95f2a20b-c7cd-4146-9931-0460a87d2b7c/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2016.rar" xr:uid="{FEB8C29C-6FD4-334D-8F74-12D9414AEFAD}"/>
+    <hyperlink ref="C52" r:id="rId39" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/079e3a33-728f-468a-b435-5ea1be346e42/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2016.rar" xr:uid="{918F7FA8-4445-BA40-9491-2E6AC84544B7}"/>
+    <hyperlink ref="C54" r:id="rId40" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/58d1a29c-7c17-4ace-86e9-552f5e4f9644/download/i_frota_por_uf_municipio_marca_e_modelo_ano_setembro_2015.rar" xr:uid="{D9506705-92A1-FA48-987D-2D08081E85F2}"/>
+    <hyperlink ref="C55" r:id="rId41" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/d0db7133-2e02-45b1-ba9f-ec9375c7250d/download/i_frota_por_uf_municipio_marca_e_modelo_ano_agosto_2015.rar" xr:uid="{871DA683-A296-7B49-93AE-6FF668332080}"/>
+    <hyperlink ref="C56" r:id="rId42" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/124c530e-7212-4026-b874-e954ae32f08a/download/i_frota_por_uf_municipio_marca_e_modelo_ano_maio_2015.rar" xr:uid="{3BEA8807-31AB-B345-BF9B-6D455A8F9A8D}"/>
+    <hyperlink ref="C57" r:id="rId43" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/30293b59-f3ed-4b7e-beac-6255a98595ff/download/i_frota_por_uf_municipio_marca_e_modelo_ano_outubro_2015.rar" xr:uid="{D0E20417-0F4B-EF47-893D-62CA80C50D9E}"/>
+    <hyperlink ref="C59" r:id="rId44" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/1ced3149-49a1-4248-bcda-75d267e56059/download/i_frota_por_uf_municipio_marca_e_modelo_ano_marco_2015.rar" xr:uid="{D9248F29-E2EC-3442-928F-4D8ED7815325}"/>
+    <hyperlink ref="C60" r:id="rId45" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/93520344-d868-4e4f-afec-a295a5b09f52/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2015.rar" xr:uid="{67F18216-7680-AB49-B5FE-569D1FA8AD0D}"/>
+    <hyperlink ref="C61" r:id="rId46" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/f3b46afe-0ba1-452d-a04d-df23446161ca/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2014.zip" xr:uid="{07B73C55-8DA7-6F4D-9199-E73D20D4342B}"/>
+    <hyperlink ref="C63" r:id="rId47" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/73319382-e55d-422b-97fc-7127a37237a3/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2014.zip" xr:uid="{0E0D127C-3B25-284B-A195-BEC29EC9877C}"/>
+    <hyperlink ref="C65" r:id="rId48" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/5a4867ff-2453-4238-b440-885c835bc233/download/i_frota_por_uf_municipio_marca_e_modelo_ano_maio_2014.zip" xr:uid="{BC9A8E4E-AEBF-3D40-A856-36B368E6A0E7}"/>
+    <hyperlink ref="C66" r:id="rId49" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/1c199cdd-9581-4a07-a205-a7e378464717/download/i_frota_por_uf_municipio_marca_e_modelo_ano_fevereiro_2014.zip" xr:uid="{B4A42A7A-B149-4644-8E2D-77748F7BCFEB}"/>
+    <hyperlink ref="C67" r:id="rId50" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/cbcb4b9d-745d-42f7-89e4-b2eb6e55d320/download/i_frota_por_uf_municipio_marca_e_modelo_ano_janeiro_2014.zip" xr:uid="{543763BC-DAC0-6746-9C91-F2351B12BC27}"/>
+    <hyperlink ref="C68" r:id="rId51" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/086f527b-ba8c-40cf-bf37-d050978db888/download/i_frota_por_uf_municipio_marca_e_modelo_ano_dezembro_2013.zip" xr:uid="{7B49B406-BBF9-3449-B5D0-EA315FC8DEC2}"/>
+    <hyperlink ref="C69" r:id="rId52" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/1d89882c-da9e-4019-9711-c27919bb99d7/download/i_frota_por_uf_municipio_marca_e_modelo_ano_novembro_2013.zip" xr:uid="{36DF4B8B-2C67-E14E-BC44-91D8640C2BB1}"/>
+    <hyperlink ref="C70" r:id="rId53" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/60cd5ad4-d96b-46c8-9d81-30fc25cd163e/download/i_frota_por_uf_municipio_marca_e_modelo_ano_julho_2013.zip" xr:uid="{D202EEBF-FA2D-A948-8A27-AED2FEE897C0}"/>
+    <hyperlink ref="C71" r:id="rId54" tooltip="https://dados.transportes.gov.br/dataset/12686da0-3d71-4499-b432-d270f785c907/resource/e0d5ae22-bf42-447a-a788-2f6f1edf9705/download/i_frota_por_uf_municipio_marca_e_modelo_ano_maio_2013.zip" xr:uid="{D29B307C-D684-684D-B808-896574FA432D}"/>
+    <hyperlink ref="B55" r:id="rId55" xr:uid="{1A3D428E-E368-FB42-A8D4-DD387A74FB5C}"/>
+    <hyperlink ref="B56" r:id="rId56" xr:uid="{FF4AAA16-5B7E-4545-A83F-62ABEA4F564D}"/>
+    <hyperlink ref="B53" r:id="rId57" xr:uid="{445187A0-2321-B345-8CE7-817B2A3786B6}"/>
+    <hyperlink ref="B50" r:id="rId58" xr:uid="{E39AF676-7888-6B44-8408-CE0A5B8ED65B}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>